<commit_message>
July 31 2025 changes DRC job type changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0047923_TMTT0047926_TMTT0047929_1_VerifyJobTypeDisplayedInJobTypeDropDownWhileAddingNewOpportunity.xlsx
+++ b/TestData/LV_TMTT0047923_TMTT0047926_TMTT0047929_1_VerifyJobTypeDisplayedInJobTypeDropDownWhileAddingNewOpportunity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBF0C5FD-B71A-49BD-82D5-D4AA714ABBF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5C0A69-EAB7-4D78-B750-06541A21A8DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUser" sheetId="2" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="AddContact" sheetId="14" r:id="rId7"/>
     <sheet name="Engagement" sheetId="20" r:id="rId8"/>
     <sheet name="ProductTypeCode" sheetId="25" r:id="rId9"/>
+    <sheet name="EngStage" sheetId="26" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="96">
   <si>
     <t>User</t>
   </si>
@@ -326,13 +327,19 @@
   </si>
   <si>
     <t>Other FVA</t>
+  </si>
+  <si>
+    <t>Opinion Report</t>
+  </si>
+  <si>
+    <t>EngStage</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -362,6 +369,12 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF181818"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -416,7 +429,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -427,6 +440,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -740,6 +754,29 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1940DEA-807A-4278-A817-36DDB491A83A}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{204DA895-5616-4092-9340-8DD85852997B}">
   <dimension ref="A1:C3"/>

</xml_diff>

<commit_message>
Staff Role changes Sept 3 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0047923_TMTT0047926_TMTT0047929_1_VerifyJobTypeDisplayedInJobTypeDropDownWhileAddingNewOpportunity.xlsx
+++ b/TestData/LV_TMTT0047923_TMTT0047926_TMTT0047929_1_VerifyJobTypeDisplayedInJobTypeDropDownWhileAddingNewOpportunity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F8443DE-56AB-4A69-86C6-3DE0324A6598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{240B1152-0447-44FF-99E5-D27B9D00A4DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUser" sheetId="2" r:id="rId1"/>

</xml_diff>